<commit_message>
Documents: Update the thesaurus and create a Word document with the summaries of articles 1 to 10.
</commit_message>
<xml_diff>
--- a/02-week/02-session/02-activity/Thesaurus_carlos.xlsx
+++ b/02-week/02-session/02-activity/Thesaurus_carlos.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EQUIPO\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Apache24\htdocs\ADSO-2899747\02-week\02-session\02-activity\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC691CEA-2A8C-44E8-A5B0-92E769422CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ANEXO" sheetId="4" r:id="rId1"/>
@@ -256,7 +257,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -390,7 +391,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -476,34 +477,22 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -826,20 +815,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G92"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="33.42578125" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" customWidth="1"/>
-    <col min="4" max="4" width="44.85546875" customWidth="1"/>
-    <col min="5" max="5" width="27.7109375" style="20" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="33.44140625" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" customWidth="1"/>
+    <col min="4" max="4" width="44.88671875" customWidth="1"/>
+    <col min="5" max="5" width="27.6640625" style="20" customWidth="1"/>
     <col min="6" max="6" width="57" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>7</v>
       </c>
@@ -862,14 +851,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="36">
+      <c r="C2" s="1">
         <v>2018</v>
       </c>
       <c r="D2" s="21" t="s">
@@ -885,37 +874,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="36">
+      <c r="C3" s="1">
         <v>2015</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="31" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="35" t="s">
+      <c r="E3" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="36">
+      <c r="C4" s="1">
         <v>2016</v>
       </c>
       <c r="D4" s="25" t="s">
@@ -931,14 +920,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="36">
+      <c r="C5" s="1">
         <v>2016</v>
       </c>
       <c r="D5" s="28" t="s">
@@ -954,14 +943,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="36">
+      <c r="C6" s="1">
         <v>2016</v>
       </c>
       <c r="D6" s="28" t="s">
@@ -977,14 +966,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="1">
         <v>2025</v>
       </c>
       <c r="D7" s="28" t="s">
@@ -1000,14 +989,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="36">
+      <c r="C8" s="1">
         <v>2025</v>
       </c>
       <c r="D8" s="25" t="s">
@@ -1023,14 +1012,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="36">
+      <c r="C9" s="1">
         <v>2015</v>
       </c>
       <c r="D9" s="25" t="s">
@@ -1046,37 +1035,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="240" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="216" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="36">
+      <c r="C10" s="1">
         <v>2022</v>
       </c>
-      <c r="D10" s="30" t="s">
+      <c r="D10" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="E10" s="31" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" s="32" t="s">
+      <c r="E10" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="31" t="s">
+      <c r="G10" s="30" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="36">
+      <c r="C11" s="1">
         <v>2021</v>
       </c>
       <c r="D11" s="28" t="s">
@@ -1092,14 +1081,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="36">
+      <c r="C12" s="1">
         <v>2024</v>
       </c>
       <c r="D12" s="28" t="s">
@@ -1115,14 +1104,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="36">
+      <c r="C13" s="1">
         <v>2023</v>
       </c>
       <c r="D13" s="25" t="s">
@@ -1138,14 +1127,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="36">
+      <c r="C14" s="1">
         <v>2022</v>
       </c>
       <c r="D14" s="28" t="s">
@@ -1161,14 +1150,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="36">
+      <c r="C15" s="1">
         <v>2022</v>
       </c>
       <c r="D15" s="28" t="s">
@@ -1184,14 +1173,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
       <c r="B16" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="36">
+      <c r="C16" s="1">
         <v>2024</v>
       </c>
       <c r="D16" s="28" t="s">
@@ -1207,14 +1196,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
       <c r="B17" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="36">
+      <c r="C17" s="1">
         <v>2022</v>
       </c>
       <c r="D17" s="25" t="s">
@@ -1230,14 +1219,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
       <c r="B18" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="C18" s="36">
+      <c r="C18" s="1">
         <v>2022</v>
       </c>
       <c r="D18" s="25" t="s">
@@ -1253,14 +1242,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
       <c r="B19" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="36">
+      <c r="C19" s="1">
         <v>2022</v>
       </c>
       <c r="D19" s="25" t="s">
@@ -1276,14 +1265,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
       <c r="B20" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C20" s="37">
+      <c r="C20" s="33">
         <v>2021</v>
       </c>
       <c r="D20" s="25" t="s">
@@ -1299,17 +1288,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="39" t="s">
+      <c r="B21" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="36">
+      <c r="C21" s="1">
         <v>2023</v>
       </c>
-      <c r="D21" s="40" t="s">
+      <c r="D21" s="36" t="s">
         <v>62</v>
       </c>
       <c r="E21" s="1" t="s">
@@ -1322,16 +1311,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="6"/>
-      <c r="C22" s="38"/>
+      <c r="C22" s="34"/>
       <c r="D22" s="8"/>
       <c r="E22" s="18"/>
       <c r="F22" s="9"/>
       <c r="G22" s="10"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="6"/>
       <c r="C23" s="7"/>
@@ -1340,7 +1329,7 @@
       <c r="F23" s="9"/>
       <c r="G23" s="10"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" s="12"/>
       <c r="C24" s="5"/>
@@ -1349,7 +1338,7 @@
       <c r="F24" s="14"/>
       <c r="G24" s="10"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
       <c r="B25" s="12"/>
       <c r="C25" s="5"/>
@@ -1358,7 +1347,7 @@
       <c r="F25" s="14"/>
       <c r="G25" s="10"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="6"/>
       <c r="C26" s="7"/>
@@ -1367,7 +1356,7 @@
       <c r="F26" s="9"/>
       <c r="G26" s="15"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="6"/>
       <c r="C27" s="7"/>
@@ -1376,7 +1365,7 @@
       <c r="F27" s="9"/>
       <c r="G27" s="10"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7"/>
@@ -1385,7 +1374,7 @@
       <c r="F28" s="9"/>
       <c r="G28" s="15"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="6"/>
       <c r="C29" s="7"/>
@@ -1394,7 +1383,7 @@
       <c r="F29" s="9"/>
       <c r="G29" s="15"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="5"/>
       <c r="B30" s="6"/>
       <c r="C30" s="7"/>
@@ -1403,7 +1392,7 @@
       <c r="F30" s="9"/>
       <c r="G30" s="15"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="5"/>
       <c r="B31" s="12"/>
       <c r="C31" s="5"/>
@@ -1412,7 +1401,7 @@
       <c r="F31" s="14"/>
       <c r="G31" s="10"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="5"/>
       <c r="B32" s="12"/>
       <c r="C32" s="5"/>
@@ -1421,7 +1410,7 @@
       <c r="F32" s="14"/>
       <c r="G32" s="10"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="5"/>
       <c r="B33" s="12"/>
       <c r="C33" s="5"/>
@@ -1430,7 +1419,7 @@
       <c r="F33" s="14"/>
       <c r="G33" s="10"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="5"/>
       <c r="B34" s="12"/>
       <c r="C34" s="5"/>
@@ -1439,7 +1428,7 @@
       <c r="F34" s="14"/>
       <c r="G34" s="10"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="5"/>
       <c r="B35" s="12"/>
       <c r="C35" s="5"/>
@@ -1448,7 +1437,7 @@
       <c r="F35" s="14"/>
       <c r="G35" s="10"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="5"/>
       <c r="B36" s="12"/>
       <c r="C36" s="7"/>
@@ -1457,7 +1446,7 @@
       <c r="F36" s="9"/>
       <c r="G36" s="10"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="5"/>
       <c r="B37" s="6"/>
       <c r="C37" s="7"/>
@@ -1466,7 +1455,7 @@
       <c r="F37" s="9"/>
       <c r="G37" s="15"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="5"/>
       <c r="B38" s="12"/>
       <c r="C38" s="7"/>
@@ -1475,7 +1464,7 @@
       <c r="F38" s="17"/>
       <c r="G38" s="10"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="5"/>
       <c r="B39" s="12"/>
       <c r="C39" s="7"/>
@@ -1484,7 +1473,7 @@
       <c r="F39" s="9"/>
       <c r="G39" s="10"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="5"/>
       <c r="B40" s="6"/>
       <c r="C40" s="7"/>
@@ -1493,7 +1482,7 @@
       <c r="F40" s="9"/>
       <c r="G40" s="15"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="5"/>
       <c r="B41" s="6"/>
       <c r="C41" s="7"/>
@@ -1502,7 +1491,7 @@
       <c r="F41" s="9"/>
       <c r="G41" s="15"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="5"/>
       <c r="B42" s="6"/>
       <c r="C42" s="7"/>
@@ -1511,7 +1500,7 @@
       <c r="F42" s="9"/>
       <c r="G42" s="15"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="5"/>
       <c r="B43" s="6"/>
       <c r="C43" s="7"/>
@@ -1520,7 +1509,7 @@
       <c r="F43" s="9"/>
       <c r="G43" s="15"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="5"/>
       <c r="B44" s="6"/>
       <c r="C44" s="7"/>
@@ -1529,7 +1518,7 @@
       <c r="F44" s="9"/>
       <c r="G44" s="15"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="5"/>
       <c r="B45" s="6"/>
       <c r="C45" s="7"/>
@@ -1538,7 +1527,7 @@
       <c r="F45" s="9"/>
       <c r="G45" s="15"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="5"/>
       <c r="B46" s="6"/>
       <c r="C46" s="7"/>
@@ -1547,7 +1536,7 @@
       <c r="F46" s="9"/>
       <c r="G46" s="15"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="5"/>
       <c r="B47" s="12"/>
       <c r="C47" s="5"/>
@@ -1556,7 +1545,7 @@
       <c r="F47" s="14"/>
       <c r="G47" s="10"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="5"/>
       <c r="B48" s="6"/>
       <c r="C48" s="7"/>
@@ -1565,7 +1554,7 @@
       <c r="F48" s="9"/>
       <c r="G48" s="15"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="5"/>
       <c r="B49" s="6"/>
       <c r="C49" s="7"/>
@@ -1574,7 +1563,7 @@
       <c r="F49" s="9"/>
       <c r="G49" s="15"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="5"/>
       <c r="B50" s="6"/>
       <c r="C50" s="7"/>
@@ -1583,7 +1572,7 @@
       <c r="F50" s="9"/>
       <c r="G50" s="15"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="5"/>
       <c r="B51" s="6"/>
       <c r="C51" s="7"/>
@@ -1592,7 +1581,7 @@
       <c r="F51" s="9"/>
       <c r="G51" s="15"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="5"/>
       <c r="B52" s="6"/>
       <c r="C52" s="7"/>
@@ -1601,7 +1590,7 @@
       <c r="F52" s="9"/>
       <c r="G52" s="15"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="5"/>
       <c r="B53" s="6"/>
       <c r="C53" s="7"/>
@@ -1610,7 +1599,7 @@
       <c r="F53" s="9"/>
       <c r="G53" s="15"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="5"/>
       <c r="B54" s="6"/>
       <c r="C54" s="7"/>
@@ -1619,7 +1608,7 @@
       <c r="F54" s="9"/>
       <c r="G54" s="15"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="5"/>
       <c r="B55" s="6"/>
       <c r="C55" s="7"/>
@@ -1628,7 +1617,7 @@
       <c r="F55" s="9"/>
       <c r="G55" s="15"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="5"/>
       <c r="B56" s="12"/>
       <c r="C56" s="5"/>
@@ -1637,7 +1626,7 @@
       <c r="F56" s="14"/>
       <c r="G56" s="10"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="5"/>
       <c r="B57" s="12"/>
       <c r="C57" s="5"/>
@@ -1646,7 +1635,7 @@
       <c r="F57" s="14"/>
       <c r="G57" s="10"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="5"/>
       <c r="B58" s="6"/>
       <c r="C58" s="7"/>
@@ -1655,7 +1644,7 @@
       <c r="F58" s="9"/>
       <c r="G58" s="10"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="5"/>
       <c r="B59" s="6"/>
       <c r="C59" s="7"/>
@@ -1663,7 +1652,7 @@
       <c r="E59" s="5"/>
       <c r="F59" s="9"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="5"/>
       <c r="B60" s="6"/>
       <c r="C60" s="7"/>
@@ -1672,7 +1661,7 @@
       <c r="F60" s="9"/>
       <c r="G60" s="10"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="5"/>
       <c r="B61" s="6"/>
       <c r="C61" s="7"/>
@@ -1681,7 +1670,7 @@
       <c r="F61" s="9"/>
       <c r="G61" s="15"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="5"/>
       <c r="B62" s="6"/>
       <c r="C62" s="7"/>
@@ -1690,7 +1679,7 @@
       <c r="F62" s="9"/>
       <c r="G62" s="15"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="5"/>
       <c r="B63" s="6"/>
       <c r="C63" s="7"/>
@@ -1699,7 +1688,7 @@
       <c r="F63" s="9"/>
       <c r="G63" s="15"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="5"/>
       <c r="B64" s="6"/>
       <c r="C64" s="7"/>
@@ -1708,7 +1697,7 @@
       <c r="F64" s="9"/>
       <c r="G64" s="15"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="5"/>
       <c r="B65" s="6"/>
       <c r="C65" s="7"/>
@@ -1717,7 +1706,7 @@
       <c r="F65" s="9"/>
       <c r="G65" s="15"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="5"/>
       <c r="B66" s="6"/>
       <c r="C66" s="7"/>
@@ -1726,7 +1715,7 @@
       <c r="F66" s="9"/>
       <c r="G66" s="15"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="5"/>
       <c r="B67" s="6"/>
       <c r="C67" s="7"/>
@@ -1735,7 +1724,7 @@
       <c r="F67" s="9"/>
       <c r="G67" s="15"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="5"/>
       <c r="B68" s="6"/>
       <c r="C68" s="7"/>
@@ -1744,7 +1733,7 @@
       <c r="F68" s="9"/>
       <c r="G68" s="15"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="5"/>
       <c r="B69" s="6"/>
       <c r="C69" s="7"/>
@@ -1753,7 +1742,7 @@
       <c r="F69" s="9"/>
       <c r="G69" s="10"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="5"/>
       <c r="B70" s="6"/>
       <c r="C70" s="7"/>
@@ -1762,7 +1751,7 @@
       <c r="F70" s="9"/>
       <c r="G70" s="10"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="5"/>
       <c r="B71" s="6"/>
       <c r="C71" s="7"/>
@@ -1771,7 +1760,7 @@
       <c r="F71" s="9"/>
       <c r="G71" s="15"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="5"/>
       <c r="B72" s="6"/>
       <c r="C72" s="7"/>
@@ -1780,7 +1769,7 @@
       <c r="F72" s="9"/>
       <c r="G72" s="15"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="5"/>
       <c r="B73" s="6"/>
       <c r="C73" s="7"/>
@@ -1789,7 +1778,7 @@
       <c r="F73" s="9"/>
       <c r="G73" s="15"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="5"/>
       <c r="B74" s="12"/>
       <c r="C74" s="5"/>
@@ -1798,7 +1787,7 @@
       <c r="F74" s="14"/>
       <c r="G74" s="10"/>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="5"/>
       <c r="B75" s="12"/>
       <c r="C75" s="5"/>
@@ -1807,7 +1796,7 @@
       <c r="F75" s="14"/>
       <c r="G75" s="10"/>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="5"/>
       <c r="B76" s="12"/>
       <c r="C76" s="5"/>
@@ -1816,7 +1805,7 @@
       <c r="F76" s="14"/>
       <c r="G76" s="10"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="5"/>
       <c r="B77" s="12"/>
       <c r="C77" s="5"/>
@@ -1825,7 +1814,7 @@
       <c r="F77" s="14"/>
       <c r="G77" s="10"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="5"/>
       <c r="B78" s="12"/>
       <c r="C78" s="5"/>
@@ -1834,7 +1823,7 @@
       <c r="F78" s="14"/>
       <c r="G78" s="10"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="5"/>
       <c r="B79" s="6"/>
       <c r="C79" s="7"/>
@@ -1843,7 +1832,7 @@
       <c r="F79" s="9"/>
       <c r="G79" s="15"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" s="5"/>
       <c r="B80" s="6"/>
       <c r="C80" s="7"/>
@@ -1852,7 +1841,7 @@
       <c r="F80" s="9"/>
       <c r="G80" s="15"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" s="5"/>
       <c r="B81" s="6"/>
       <c r="C81" s="7"/>
@@ -1861,7 +1850,7 @@
       <c r="F81" s="9"/>
       <c r="G81" s="15"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="5"/>
       <c r="B82" s="6"/>
       <c r="C82" s="7"/>
@@ -1870,7 +1859,7 @@
       <c r="F82" s="9"/>
       <c r="G82" s="15"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="5"/>
       <c r="B83" s="6"/>
       <c r="C83" s="7"/>
@@ -1879,7 +1868,7 @@
       <c r="F83" s="9"/>
       <c r="G83" s="15"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="5"/>
       <c r="B84" s="6"/>
       <c r="C84" s="7"/>
@@ -1888,7 +1877,7 @@
       <c r="F84" s="9"/>
       <c r="G84" s="15"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" s="5"/>
       <c r="B85" s="6"/>
       <c r="C85" s="7"/>
@@ -1897,7 +1886,7 @@
       <c r="F85" s="9"/>
       <c r="G85" s="15"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="5"/>
       <c r="B86" s="6"/>
       <c r="C86" s="7"/>
@@ -1906,7 +1895,7 @@
       <c r="F86" s="9"/>
       <c r="G86" s="15"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" s="5"/>
       <c r="B87" s="6"/>
       <c r="C87" s="7"/>
@@ -1915,7 +1904,7 @@
       <c r="F87" s="9"/>
       <c r="G87" s="15"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" s="5"/>
       <c r="B88" s="6"/>
       <c r="C88" s="7"/>
@@ -1924,7 +1913,7 @@
       <c r="F88" s="9"/>
       <c r="G88" s="15"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" s="5"/>
       <c r="B89" s="6"/>
       <c r="C89" s="7"/>
@@ -1933,7 +1922,7 @@
       <c r="F89" s="9"/>
       <c r="G89" s="15"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" s="5"/>
       <c r="B90" s="6"/>
       <c r="C90" s="7"/>
@@ -1942,7 +1931,7 @@
       <c r="F90" s="9"/>
       <c r="G90" s="15"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" s="5"/>
       <c r="B91" s="6"/>
       <c r="C91" s="7"/>
@@ -1951,7 +1940,7 @@
       <c r="F91" s="9"/>
       <c r="G91" s="15"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" s="5"/>
       <c r="B92" s="6"/>
       <c r="C92" s="7"/>
@@ -1961,31 +1950,31 @@
       <c r="G92" s="15"/>
     </row>
   </sheetData>
-  <sortState ref="A2:G92">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G92">
     <sortCondition ref="G2:G92"/>
     <sortCondition ref="B2:B92"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1"/>
-    <hyperlink ref="D4" r:id="rId2"/>
-    <hyperlink ref="D5" r:id="rId3"/>
-    <hyperlink ref="D6" r:id="rId4"/>
-    <hyperlink ref="D7" r:id="rId5"/>
-    <hyperlink ref="D8" r:id="rId6"/>
-    <hyperlink ref="D9" r:id="rId7"/>
-    <hyperlink ref="D10"/>
-    <hyperlink ref="D11" r:id="rId8"/>
-    <hyperlink ref="D12" r:id="rId9"/>
-    <hyperlink ref="D13" r:id="rId10"/>
-    <hyperlink ref="D14" r:id="rId11"/>
-    <hyperlink ref="D15" r:id="rId12"/>
-    <hyperlink ref="D16" r:id="rId13"/>
-    <hyperlink ref="D17" r:id="rId14"/>
-    <hyperlink ref="D18" r:id="rId15"/>
-    <hyperlink ref="D19" r:id="rId16"/>
-    <hyperlink ref="D20" r:id="rId17"/>
-    <hyperlink ref="D21" r:id="rId18"/>
-    <hyperlink ref="D3" r:id="rId19"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="D7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="D8" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="D9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="D10" display="https://d1wqtxts1xzle7.cloudfront.net/111860414/18841-libre.pdf?1708974048=&amp;response-content-disposition=inline%3B+filename%3DEasyRest_Generador_automatico_de_API_Res.pdf&amp;Expires=1756126855&amp;Signature=PfW2C2QHi7Wp4BuhUwi0rQpjIJgRsm1r7NunpWEpVpdoZ~FzGJeMnHs" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D11" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="D12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="D13" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="D14" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="D15" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="D16" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="D17" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="D18" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="D19" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="D20" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="D21" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="D3" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: add research article on UrbanTracker project
</commit_message>
<xml_diff>
--- a/02-week/02-session/02-activity/Thesaurus_carlos.xlsx
+++ b/02-week/02-session/02-activity/Thesaurus_carlos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Apache24\htdocs\ADSO-2899747\02-week\02-session\02-activity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC691CEA-2A8C-44E8-A5B0-92E769422CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF138A99-4444-4D7F-9D80-7592D3A259E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ANEXO" sheetId="4" r:id="rId1"/>
@@ -86,10 +86,6 @@
     <t>https://web.archive.org/web/20180415091800id_/http://revistas.usc.edu.co/index.php/Ingenium/article/viewFile/651/518</t>
   </si>
   <si>
-    <t xml:space="preserve">SisMo: sistema de seguridad para motocicletas 
-</t>
-  </si>
-  <si>
     <t xml:space="preserve"> "articulos"  and "gps" and "mqtt" and "java"</t>
   </si>
   <si>
@@ -252,6 +248,9 @@
   </si>
   <si>
     <t>https://ciencialatina.org/index.php/cienciala/article/view/2959/4350</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SisMo: sistema de seguridad para motocicletas </t>
   </si>
 </sst>
 </file>
@@ -817,18 +816,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G92"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" customWidth="1"/>
-    <col min="2" max="2" width="33.44140625" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" customWidth="1"/>
-    <col min="4" max="4" width="44.88671875" customWidth="1"/>
-    <col min="5" max="5" width="27.6640625" style="20" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" customWidth="1"/>
+    <col min="2" max="2" width="33.42578125" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" customWidth="1"/>
+    <col min="4" max="4" width="44.85546875" customWidth="1"/>
+    <col min="5" max="5" width="27.7109375" style="20" customWidth="1"/>
     <col min="6" max="6" width="57" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>7</v>
       </c>
@@ -851,12 +850,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C2" s="1">
         <v>2018</v>
@@ -874,30 +873,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" s="1">
         <v>2015</v>
       </c>
       <c r="D3" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E3" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -920,7 +919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -943,12 +942,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1">
         <v>2016</v>
@@ -960,358 +959,358 @@
         <v>8</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7" s="1">
         <v>2025</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C8" s="1">
         <v>2025</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C9" s="1">
         <v>2015</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="216" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="240" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="1">
         <v>2022</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E10" s="30" t="s">
         <v>8</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G10" s="30" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C11" s="1">
         <v>2021</v>
       </c>
       <c r="D11" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="22" t="s">
         <v>31</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11" s="22" t="s">
-        <v>32</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C12" s="1">
         <v>2024</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" s="1">
         <v>2023</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C14" s="1">
         <v>2022</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F14" s="22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" s="1">
         <v>2022</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C16" s="1">
         <v>2024</v>
       </c>
       <c r="D16" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="22" t="s">
         <v>47</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F16" s="22" t="s">
-        <v>48</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C17" s="1">
         <v>2022</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F17" s="22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C18" s="1">
         <v>2022</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F18" s="22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>18</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C19" s="1">
         <v>2022</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C20" s="33">
         <v>2021</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
       <c r="B21" s="35" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C21" s="1">
         <v>2023</v>
       </c>
       <c r="D21" s="36" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="B22" s="6"/>
       <c r="C22" s="34"/>
@@ -1320,7 +1319,7 @@
       <c r="F22" s="9"/>
       <c r="G22" s="10"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
       <c r="B23" s="6"/>
       <c r="C23" s="7"/>
@@ -1329,7 +1328,7 @@
       <c r="F23" s="9"/>
       <c r="G23" s="10"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" s="12"/>
       <c r="C24" s="5"/>
@@ -1338,7 +1337,7 @@
       <c r="F24" s="14"/>
       <c r="G24" s="10"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="5"/>
       <c r="B25" s="12"/>
       <c r="C25" s="5"/>
@@ -1347,7 +1346,7 @@
       <c r="F25" s="14"/>
       <c r="G25" s="10"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
       <c r="B26" s="6"/>
       <c r="C26" s="7"/>
@@ -1356,7 +1355,7 @@
       <c r="F26" s="9"/>
       <c r="G26" s="15"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="5"/>
       <c r="B27" s="6"/>
       <c r="C27" s="7"/>
@@ -1365,7 +1364,7 @@
       <c r="F27" s="9"/>
       <c r="G27" s="10"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="5"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7"/>
@@ -1374,7 +1373,7 @@
       <c r="F28" s="9"/>
       <c r="G28" s="15"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
       <c r="B29" s="6"/>
       <c r="C29" s="7"/>
@@ -1383,7 +1382,7 @@
       <c r="F29" s="9"/>
       <c r="G29" s="15"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
       <c r="B30" s="6"/>
       <c r="C30" s="7"/>
@@ -1392,7 +1391,7 @@
       <c r="F30" s="9"/>
       <c r="G30" s="15"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
       <c r="B31" s="12"/>
       <c r="C31" s="5"/>
@@ -1401,7 +1400,7 @@
       <c r="F31" s="14"/>
       <c r="G31" s="10"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="5"/>
       <c r="B32" s="12"/>
       <c r="C32" s="5"/>
@@ -1410,7 +1409,7 @@
       <c r="F32" s="14"/>
       <c r="G32" s="10"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
       <c r="B33" s="12"/>
       <c r="C33" s="5"/>
@@ -1419,7 +1418,7 @@
       <c r="F33" s="14"/>
       <c r="G33" s="10"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="5"/>
       <c r="B34" s="12"/>
       <c r="C34" s="5"/>
@@ -1428,7 +1427,7 @@
       <c r="F34" s="14"/>
       <c r="G34" s="10"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="5"/>
       <c r="B35" s="12"/>
       <c r="C35" s="5"/>
@@ -1437,7 +1436,7 @@
       <c r="F35" s="14"/>
       <c r="G35" s="10"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="5"/>
       <c r="B36" s="12"/>
       <c r="C36" s="7"/>
@@ -1446,7 +1445,7 @@
       <c r="F36" s="9"/>
       <c r="G36" s="10"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="5"/>
       <c r="B37" s="6"/>
       <c r="C37" s="7"/>
@@ -1455,7 +1454,7 @@
       <c r="F37" s="9"/>
       <c r="G37" s="15"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="5"/>
       <c r="B38" s="12"/>
       <c r="C38" s="7"/>
@@ -1464,7 +1463,7 @@
       <c r="F38" s="17"/>
       <c r="G38" s="10"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="5"/>
       <c r="B39" s="12"/>
       <c r="C39" s="7"/>
@@ -1473,7 +1472,7 @@
       <c r="F39" s="9"/>
       <c r="G39" s="10"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="5"/>
       <c r="B40" s="6"/>
       <c r="C40" s="7"/>
@@ -1482,7 +1481,7 @@
       <c r="F40" s="9"/>
       <c r="G40" s="15"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="5"/>
       <c r="B41" s="6"/>
       <c r="C41" s="7"/>
@@ -1491,7 +1490,7 @@
       <c r="F41" s="9"/>
       <c r="G41" s="15"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="5"/>
       <c r="B42" s="6"/>
       <c r="C42" s="7"/>
@@ -1500,7 +1499,7 @@
       <c r="F42" s="9"/>
       <c r="G42" s="15"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="5"/>
       <c r="B43" s="6"/>
       <c r="C43" s="7"/>
@@ -1509,7 +1508,7 @@
       <c r="F43" s="9"/>
       <c r="G43" s="15"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="5"/>
       <c r="B44" s="6"/>
       <c r="C44" s="7"/>
@@ -1518,7 +1517,7 @@
       <c r="F44" s="9"/>
       <c r="G44" s="15"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="5"/>
       <c r="B45" s="6"/>
       <c r="C45" s="7"/>
@@ -1527,7 +1526,7 @@
       <c r="F45" s="9"/>
       <c r="G45" s="15"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="5"/>
       <c r="B46" s="6"/>
       <c r="C46" s="7"/>
@@ -1536,7 +1535,7 @@
       <c r="F46" s="9"/>
       <c r="G46" s="15"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="5"/>
       <c r="B47" s="12"/>
       <c r="C47" s="5"/>
@@ -1545,7 +1544,7 @@
       <c r="F47" s="14"/>
       <c r="G47" s="10"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="5"/>
       <c r="B48" s="6"/>
       <c r="C48" s="7"/>
@@ -1554,7 +1553,7 @@
       <c r="F48" s="9"/>
       <c r="G48" s="15"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="5"/>
       <c r="B49" s="6"/>
       <c r="C49" s="7"/>
@@ -1563,7 +1562,7 @@
       <c r="F49" s="9"/>
       <c r="G49" s="15"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="5"/>
       <c r="B50" s="6"/>
       <c r="C50" s="7"/>
@@ -1572,7 +1571,7 @@
       <c r="F50" s="9"/>
       <c r="G50" s="15"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="5"/>
       <c r="B51" s="6"/>
       <c r="C51" s="7"/>
@@ -1581,7 +1580,7 @@
       <c r="F51" s="9"/>
       <c r="G51" s="15"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="5"/>
       <c r="B52" s="6"/>
       <c r="C52" s="7"/>
@@ -1590,7 +1589,7 @@
       <c r="F52" s="9"/>
       <c r="G52" s="15"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="5"/>
       <c r="B53" s="6"/>
       <c r="C53" s="7"/>
@@ -1599,7 +1598,7 @@
       <c r="F53" s="9"/>
       <c r="G53" s="15"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="5"/>
       <c r="B54" s="6"/>
       <c r="C54" s="7"/>
@@ -1608,7 +1607,7 @@
       <c r="F54" s="9"/>
       <c r="G54" s="15"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="5"/>
       <c r="B55" s="6"/>
       <c r="C55" s="7"/>
@@ -1617,7 +1616,7 @@
       <c r="F55" s="9"/>
       <c r="G55" s="15"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="5"/>
       <c r="B56" s="12"/>
       <c r="C56" s="5"/>
@@ -1626,7 +1625,7 @@
       <c r="F56" s="14"/>
       <c r="G56" s="10"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="5"/>
       <c r="B57" s="12"/>
       <c r="C57" s="5"/>
@@ -1635,7 +1634,7 @@
       <c r="F57" s="14"/>
       <c r="G57" s="10"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="5"/>
       <c r="B58" s="6"/>
       <c r="C58" s="7"/>
@@ -1644,7 +1643,7 @@
       <c r="F58" s="9"/>
       <c r="G58" s="10"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="5"/>
       <c r="B59" s="6"/>
       <c r="C59" s="7"/>
@@ -1652,7 +1651,7 @@
       <c r="E59" s="5"/>
       <c r="F59" s="9"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="5"/>
       <c r="B60" s="6"/>
       <c r="C60" s="7"/>
@@ -1661,7 +1660,7 @@
       <c r="F60" s="9"/>
       <c r="G60" s="10"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="5"/>
       <c r="B61" s="6"/>
       <c r="C61" s="7"/>
@@ -1670,7 +1669,7 @@
       <c r="F61" s="9"/>
       <c r="G61" s="15"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="5"/>
       <c r="B62" s="6"/>
       <c r="C62" s="7"/>
@@ -1679,7 +1678,7 @@
       <c r="F62" s="9"/>
       <c r="G62" s="15"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="5"/>
       <c r="B63" s="6"/>
       <c r="C63" s="7"/>
@@ -1688,7 +1687,7 @@
       <c r="F63" s="9"/>
       <c r="G63" s="15"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="5"/>
       <c r="B64" s="6"/>
       <c r="C64" s="7"/>
@@ -1697,7 +1696,7 @@
       <c r="F64" s="9"/>
       <c r="G64" s="15"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="5"/>
       <c r="B65" s="6"/>
       <c r="C65" s="7"/>
@@ -1706,7 +1705,7 @@
       <c r="F65" s="9"/>
       <c r="G65" s="15"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="5"/>
       <c r="B66" s="6"/>
       <c r="C66" s="7"/>
@@ -1715,7 +1714,7 @@
       <c r="F66" s="9"/>
       <c r="G66" s="15"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="5"/>
       <c r="B67" s="6"/>
       <c r="C67" s="7"/>
@@ -1724,7 +1723,7 @@
       <c r="F67" s="9"/>
       <c r="G67" s="15"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="5"/>
       <c r="B68" s="6"/>
       <c r="C68" s="7"/>
@@ -1733,7 +1732,7 @@
       <c r="F68" s="9"/>
       <c r="G68" s="15"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="5"/>
       <c r="B69" s="6"/>
       <c r="C69" s="7"/>
@@ -1742,7 +1741,7 @@
       <c r="F69" s="9"/>
       <c r="G69" s="10"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="5"/>
       <c r="B70" s="6"/>
       <c r="C70" s="7"/>
@@ -1751,7 +1750,7 @@
       <c r="F70" s="9"/>
       <c r="G70" s="10"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="5"/>
       <c r="B71" s="6"/>
       <c r="C71" s="7"/>
@@ -1760,7 +1759,7 @@
       <c r="F71" s="9"/>
       <c r="G71" s="15"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="5"/>
       <c r="B72" s="6"/>
       <c r="C72" s="7"/>
@@ -1769,7 +1768,7 @@
       <c r="F72" s="9"/>
       <c r="G72" s="15"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="5"/>
       <c r="B73" s="6"/>
       <c r="C73" s="7"/>
@@ -1778,7 +1777,7 @@
       <c r="F73" s="9"/>
       <c r="G73" s="15"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="5"/>
       <c r="B74" s="12"/>
       <c r="C74" s="5"/>
@@ -1787,7 +1786,7 @@
       <c r="F74" s="14"/>
       <c r="G74" s="10"/>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="5"/>
       <c r="B75" s="12"/>
       <c r="C75" s="5"/>
@@ -1796,7 +1795,7 @@
       <c r="F75" s="14"/>
       <c r="G75" s="10"/>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="5"/>
       <c r="B76" s="12"/>
       <c r="C76" s="5"/>
@@ -1805,7 +1804,7 @@
       <c r="F76" s="14"/>
       <c r="G76" s="10"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="5"/>
       <c r="B77" s="12"/>
       <c r="C77" s="5"/>
@@ -1814,7 +1813,7 @@
       <c r="F77" s="14"/>
       <c r="G77" s="10"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="5"/>
       <c r="B78" s="12"/>
       <c r="C78" s="5"/>
@@ -1823,7 +1822,7 @@
       <c r="F78" s="14"/>
       <c r="G78" s="10"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="5"/>
       <c r="B79" s="6"/>
       <c r="C79" s="7"/>
@@ -1832,7 +1831,7 @@
       <c r="F79" s="9"/>
       <c r="G79" s="15"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="5"/>
       <c r="B80" s="6"/>
       <c r="C80" s="7"/>
@@ -1841,7 +1840,7 @@
       <c r="F80" s="9"/>
       <c r="G80" s="15"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="5"/>
       <c r="B81" s="6"/>
       <c r="C81" s="7"/>
@@ -1850,7 +1849,7 @@
       <c r="F81" s="9"/>
       <c r="G81" s="15"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="5"/>
       <c r="B82" s="6"/>
       <c r="C82" s="7"/>
@@ -1859,7 +1858,7 @@
       <c r="F82" s="9"/>
       <c r="G82" s="15"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="5"/>
       <c r="B83" s="6"/>
       <c r="C83" s="7"/>
@@ -1868,7 +1867,7 @@
       <c r="F83" s="9"/>
       <c r="G83" s="15"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="5"/>
       <c r="B84" s="6"/>
       <c r="C84" s="7"/>
@@ -1877,7 +1876,7 @@
       <c r="F84" s="9"/>
       <c r="G84" s="15"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="5"/>
       <c r="B85" s="6"/>
       <c r="C85" s="7"/>
@@ -1886,7 +1885,7 @@
       <c r="F85" s="9"/>
       <c r="G85" s="15"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="5"/>
       <c r="B86" s="6"/>
       <c r="C86" s="7"/>
@@ -1895,7 +1894,7 @@
       <c r="F86" s="9"/>
       <c r="G86" s="15"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="5"/>
       <c r="B87" s="6"/>
       <c r="C87" s="7"/>
@@ -1904,7 +1903,7 @@
       <c r="F87" s="9"/>
       <c r="G87" s="15"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="5"/>
       <c r="B88" s="6"/>
       <c r="C88" s="7"/>
@@ -1913,7 +1912,7 @@
       <c r="F88" s="9"/>
       <c r="G88" s="15"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="5"/>
       <c r="B89" s="6"/>
       <c r="C89" s="7"/>
@@ -1922,7 +1921,7 @@
       <c r="F89" s="9"/>
       <c r="G89" s="15"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="5"/>
       <c r="B90" s="6"/>
       <c r="C90" s="7"/>
@@ -1931,7 +1930,7 @@
       <c r="F90" s="9"/>
       <c r="G90" s="15"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="5"/>
       <c r="B91" s="6"/>
       <c r="C91" s="7"/>
@@ -1940,7 +1939,7 @@
       <c r="F91" s="9"/>
       <c r="G91" s="15"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="5"/>
       <c r="B92" s="6"/>
       <c r="C92" s="7"/>

</xml_diff>